<commit_message>
fix(xlsx): draw 3-D charts as their flat chart families
</commit_message>
<xml_diff>
--- a/packages/xlsx/test-fixtures/unsupported-charts.xlsx
+++ b/packages/xlsx/test-fixtures/unsupported-charts.xlsx
@@ -17,21 +17,17 @@
           <a:lstStyle/>
           <a:p>
             <a:r>
-              <a:t>Revenue in 3-D</a:t>
+              <a:t>Revenue on one axis twice</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
     </c:title>
-    <c:view3D>
-      <c:rotX val="15"/>
-      <c:rotY val="20"/>
-      <c:depthPercent val="100"/>
-    </c:view3D>
     <c:plotArea>
-      <c:bar3DChart>
+      <c:barChart>
         <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
+        <c:grouping val="stacked"/>
+        <c:overlap val="100"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -87,9 +83,9 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1001"/>
         <c:axId val="1002"/>
-      </c:bar3DChart>
+        <c:axId val="1002"/>
+      </c:barChart>
       <c:catAx>
         <c:axId val="1001"/>
         <c:axPos val="b"/>

</xml_diff>